<commit_message>
Add multi-year course curriculum support and custom Teaching Assistants allocation under lecture faculty with 7-sheet Excel generator, AI chatbot, and interactive UI
</commit_message>
<xml_diff>
--- a/output/ltpc_workload_calculation.xlsx
+++ b/output/ltpc_workload_calculation.xlsx
@@ -639,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S29"/>
+  <dimension ref="A1:S39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -725,35 +725,35 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>24 hrs × 1 fac = 288 dept hrs</t>
+          <t>35 hrs × 1 fac = 420 dept hrs</t>
         </is>
       </c>
       <c r="B5" s="4" t="n"/>
       <c r="C5" s="4" t="n"/>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>0 hrs × 3 fac = 0 dept hrs</t>
+          <t>8 hrs × 3 fac = 288 dept hrs</t>
         </is>
       </c>
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="n"/>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>16 hrs × 3 fac = 576 dept hrs</t>
+          <t>36 hrs × 3 fac = 1296 dept hrs</t>
         </is>
       </c>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="n"/>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>72 hrs / section / wk</t>
+          <t>167 hrs / section / wk</t>
         </is>
       </c>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="n"/>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>864 FACULTY-HOURS / WK</t>
+          <t>2004 FACULTY-HOURS / WK</t>
         </is>
       </c>
       <c r="N5" s="4" t="n"/>
@@ -761,7 +761,7 @@
       <c r="P5" s="4" t="n"/>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>~57.6 Faculty Members</t>
+          <t>~133.6 Faculty Members</t>
         </is>
       </c>
       <c r="R5" s="4" t="n"/>
@@ -877,20 +877,20 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Advanced Linear Algebra and Optimization</t>
+          <t>Python Programming Essentials</t>
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9" s="10" t="n">
         <v>2</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G9" s="10" t="n">
         <v>5</v>
@@ -905,32 +905,32 @@
         <v>3</v>
       </c>
       <c r="K9" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L9" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M9" s="10" t="n">
         <v>6</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="O9" s="10" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="Q9" s="10" t="n">
         <v>72</v>
       </c>
       <c r="R9" s="12" t="n">
-        <v>108</v>
+        <v>156</v>
       </c>
       <c r="S9" s="10" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>7.8%</t>
         </is>
       </c>
     </row>
@@ -940,24 +940,24 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>Full Stack AI Application Development</t>
+          <t>Front-End Web Development</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E10" s="13" t="n">
         <v>2</v>
       </c>
       <c r="F10" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="G10" s="13" t="n">
-        <v>5</v>
-      </c>
       <c r="H10" s="13" t="n">
         <v>1</v>
       </c>
@@ -968,32 +968,32 @@
         <v>3</v>
       </c>
       <c r="K10" s="13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L10" s="13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M10" s="13" t="n">
         <v>6</v>
       </c>
       <c r="N10" s="15" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="O10" s="13" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="P10" s="13" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="Q10" s="13" t="n">
         <v>72</v>
       </c>
       <c r="R10" s="15" t="n">
-        <v>108</v>
+        <v>144</v>
       </c>
       <c r="S10" s="13" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>7.2%</t>
         </is>
       </c>
     </row>
@@ -1003,11 +1003,11 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Algorithm Design and Analysis</t>
+          <t>Mini Project - Branch Specific</t>
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D11" s="10" t="n">
         <v>0</v>
@@ -1016,10 +1016,10 @@
         <v>2</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H11" s="10" t="n">
         <v>1</v>
@@ -1031,7 +1031,7 @@
         <v>3</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>0</v>
@@ -1040,10 +1040,10 @@
         <v>6</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="P11" s="10" t="n">
         <v>0</v>
@@ -1052,11 +1052,11 @@
         <v>72</v>
       </c>
       <c r="R11" s="12" t="n">
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="S11" s="10" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>3.6%</t>
         </is>
       </c>
     </row>
@@ -1066,23 +1066,23 @@
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Machine Learning</t>
+          <t>Design Thinking and Engineering Orientation</t>
         </is>
       </c>
       <c r="C12" s="13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E12" s="13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F12" s="13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H12" s="13" t="n">
         <v>1</v>
@@ -1094,32 +1094,32 @@
         <v>3</v>
       </c>
       <c r="K12" s="13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L12" s="13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M12" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="N12" s="15" t="n">
-        <v>9</v>
-      </c>
       <c r="O12" s="13" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="P12" s="13" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="Q12" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="15" t="n">
         <v>72</v>
       </c>
-      <c r="R12" s="15" t="n">
-        <v>108</v>
-      </c>
       <c r="S12" s="13" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>3.6%</t>
         </is>
       </c>
     </row>
@@ -1129,14 +1129,14 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>Algorithm Design and Analysis</t>
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>2</v>
@@ -1145,7 +1145,7 @@
         <v>4</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H13" s="10" t="n">
         <v>1</v>
@@ -1157,32 +1157,32 @@
         <v>3</v>
       </c>
       <c r="K13" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L13" s="10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M13" s="10" t="n">
         <v>6</v>
       </c>
       <c r="N13" s="12" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="O13" s="10" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="P13" s="10" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="Q13" s="10" t="n">
         <v>72</v>
       </c>
       <c r="R13" s="12" t="n">
-        <v>108</v>
+        <v>168</v>
       </c>
       <c r="S13" s="10" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>8.4%</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>Digital Logic and Computer Organization</t>
+          <t>Machine Learning</t>
         </is>
       </c>
       <c r="C14" s="13" t="n">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="S14" s="13" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>5.4%</t>
         </is>
       </c>
     </row>
@@ -1255,23 +1255,23 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Excluded Course</t>
+          <t>Full Stack Development</t>
         </is>
       </c>
       <c r="C15" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D15" s="10" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F15" s="10" t="n">
         <v>4</v>
       </c>
       <c r="G15" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H15" s="10" t="n">
         <v>1</v>
@@ -1283,32 +1283,32 @@
         <v>3</v>
       </c>
       <c r="K15" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L15" s="10" t="n">
         <v>0</v>
       </c>
       <c r="M15" s="10" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="N15" s="12" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="O15" s="10" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="P15" s="10" t="n">
         <v>0</v>
       </c>
       <c r="Q15" s="10" t="n">
-        <v>72</v>
+        <v>144</v>
       </c>
       <c r="R15" s="12" t="n">
-        <v>108</v>
+        <v>168</v>
       </c>
       <c r="S15" s="10" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>8.4%</t>
         </is>
       </c>
     </row>
@@ -1318,11 +1318,11 @@
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Open Elective - 1</t>
+          <t>Digital Logic and Computer Organization</t>
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" s="13" t="n">
         <v>0</v>
@@ -1331,11 +1331,11 @@
         <v>2</v>
       </c>
       <c r="F16" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="G16" s="13" t="n">
-        <v>5</v>
-      </c>
       <c r="H16" s="13" t="n">
         <v>1</v>
       </c>
@@ -1346,7 +1346,7 @@
         <v>3</v>
       </c>
       <c r="K16" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L16" s="13" t="n">
         <v>0</v>
@@ -1355,10 +1355,10 @@
         <v>6</v>
       </c>
       <c r="N16" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O16" s="13" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="P16" s="13" t="n">
         <v>0</v>
@@ -1367,286 +1367,916 @@
         <v>72</v>
       </c>
       <c r="R16" s="15" t="n">
+        <v>96</v>
+      </c>
+      <c r="S16" s="13" t="inlineStr">
+        <is>
+          <t>4.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J17" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K17" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="L17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="O17" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="P17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="10" t="n">
+        <v>72</v>
+      </c>
+      <c r="R17" s="12" t="n">
         <v>108</v>
       </c>
-      <c r="S16" s="13" t="inlineStr">
-        <is>
-          <t>12.5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="16" t="inlineStr"/>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="S17" s="10" t="inlineStr">
+        <is>
+          <t>5.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Computer Networks</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="J18" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K18" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L18" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="N18" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="O18" s="13" t="n">
+        <v>36</v>
+      </c>
+      <c r="P18" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="13" t="n">
+        <v>72</v>
+      </c>
+      <c r="R18" s="15" t="n">
+        <v>108</v>
+      </c>
+      <c r="S18" s="13" t="inlineStr">
+        <is>
+          <t>5.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Operating Systems</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K19" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="N19" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="O19" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="P19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="10" t="n">
+        <v>72</v>
+      </c>
+      <c r="R19" s="12" t="n">
+        <v>96</v>
+      </c>
+      <c r="S19" s="10" t="inlineStr">
+        <is>
+          <t>4.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Cloud Computing</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="G20" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="H20" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="J20" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K20" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L20" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="N20" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="O20" s="13" t="n">
+        <v>36</v>
+      </c>
+      <c r="P20" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="13" t="n">
+        <v>72</v>
+      </c>
+      <c r="R20" s="15" t="n">
+        <v>108</v>
+      </c>
+      <c r="S20" s="13" t="inlineStr">
+        <is>
+          <t>5.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Web and Sequence Data Mining</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="H21" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J21" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K21" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="L21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="O21" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="P21" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="10" t="n">
+        <v>72</v>
+      </c>
+      <c r="R21" s="12" t="n">
+        <v>108</v>
+      </c>
+      <c r="S21" s="10" t="inlineStr">
+        <is>
+          <t>5.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>Big Data Analytics</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="H22" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="J22" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K22" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L22" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="N22" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="O22" s="13" t="n">
+        <v>36</v>
+      </c>
+      <c r="P22" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="13" t="n">
+        <v>72</v>
+      </c>
+      <c r="R22" s="15" t="n">
+        <v>108</v>
+      </c>
+      <c r="S22" s="13" t="inlineStr">
+        <is>
+          <t>5.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Natural Language Processing</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J23" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="O23" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="P23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="10" t="n">
+        <v>72</v>
+      </c>
+      <c r="R23" s="12" t="n">
+        <v>96</v>
+      </c>
+      <c r="S23" s="10" t="inlineStr">
+        <is>
+          <t>4.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Generative and Agentic AI</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="H24" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="J24" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="N24" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="O24" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="P24" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="13" t="n">
+        <v>72</v>
+      </c>
+      <c r="R24" s="15" t="n">
+        <v>96</v>
+      </c>
+      <c r="S24" s="13" t="inlineStr">
+        <is>
+          <t>4.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>ML Ops and LLM Ops</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G25" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J25" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K25" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="L25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="N25" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="O25" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="P25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="10" t="n">
+        <v>72</v>
+      </c>
+      <c r="R25" s="12" t="n">
+        <v>96</v>
+      </c>
+      <c r="S25" s="10" t="inlineStr">
+        <is>
+          <t>4.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Reinforcement Learning</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K26" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="L26" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="N26" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="O26" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="P26" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="13" t="n">
+        <v>72</v>
+      </c>
+      <c r="R26" s="15" t="n">
+        <v>96</v>
+      </c>
+      <c r="S26" s="13" t="inlineStr">
+        <is>
+          <t>4.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="16" t="inlineStr"/>
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>TOTAL CURRICULUM WORKLOAD</t>
         </is>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C27" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="D27" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E27" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="F27" s="17" t="n">
+        <v>57</v>
+      </c>
+      <c r="G27" s="17" t="n">
+        <v>79</v>
+      </c>
+      <c r="H27" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="J27" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="L27" s="17" t="n">
         <v>24</v>
       </c>
-      <c r="D17" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="17" t="n">
-        <v>16</v>
-      </c>
-      <c r="F17" s="17" t="n">
-        <v>32</v>
-      </c>
-      <c r="G17" s="17" t="n">
-        <v>40</v>
-      </c>
-      <c r="H17" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="J17" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="K17" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="L17" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="17" t="n">
-        <v>48</v>
-      </c>
-      <c r="N17" s="17" t="n">
-        <v>72</v>
-      </c>
-      <c r="O17" s="17" t="n">
+      <c r="M27" s="17" t="n">
+        <v>108</v>
+      </c>
+      <c r="N27" s="17" t="n">
+        <v>167</v>
+      </c>
+      <c r="O27" s="17" t="n">
+        <v>420</v>
+      </c>
+      <c r="P27" s="17" t="n">
         <v>288</v>
       </c>
-      <c r="P17" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="17" t="n">
-        <v>576</v>
-      </c>
-      <c r="R17" s="17" t="n">
-        <v>864</v>
-      </c>
-      <c r="S17" s="17" t="inlineStr">
+      <c r="Q27" s="17" t="n">
+        <v>1296</v>
+      </c>
+      <c r="R27" s="17" t="n">
+        <v>2004</v>
+      </c>
+      <c r="S27" s="17" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>MATHEMATICAL FORMULAS &amp; WORKLOAD GOVERNING PRINCIPLES</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>• Section Workload Formula:</t>
         </is>
       </c>
-      <c r="E20" s="19" t="inlineStr">
-        <is>
-          <t>24*1(L hours *1 faculty) + 0*3(T hours *3 faculty) + 16*3(P hours *3 faculty) = 72 hours</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="E30" s="19" t="inlineStr">
+        <is>
+          <t>35*1(L hours *1 faculty) + 8*3(T hours *3 faculty) + 36*3(P hours *3 faculty) = 167 hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>• Department Workload Formula (12 Sections):</t>
         </is>
       </c>
-      <c r="E21" s="19" t="inlineStr">
-        <is>
-          <t>24*1*12(L hours *1 faculty*12 sections) + 0*3*12(T hours *3 faculty*12 sections) + 16*3*12(P hours *3 faculty*12 sections) = 864 hours</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="E31" s="19" t="inlineStr">
+        <is>
+          <t>35*1*12(L hours *1 faculty*12 sections) + 8*3*12(T hours *3 faculty*12 sections) + 36*3*12(P hours *3 faculty*12 sections) = 2004 hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>• Institutional Multiplier Rule:</t>
         </is>
       </c>
-      <c r="E22" s="19" t="inlineStr">
+      <c r="E32" s="19" t="inlineStr">
         <is>
           <t>Each Lecture (L) hour has 1 faculty. Each Tutorial (T) hour has 3 faculty allotted. Each Practical (P) hour has 3 faculty allotted per section.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>• Faculty Count Requirement:</t>
         </is>
       </c>
-      <c r="E23" s="19" t="inlineStr">
-        <is>
-          <t>Total Department Workload (864 hrs) ÷ Standard Capacity (15.0 hrs/fac) = ~57.6 Faculty Members needed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="E33" s="19" t="inlineStr">
+        <is>
+          <t>Total Department Workload (2004 hrs) ÷ Standard Capacity (15.0 hrs/fac) = ~133.6 Faculty Members needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>WORKLOAD EFFICIENCY &amp; CAPACITY UTILIZATION SUMMARY</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="20" t="inlineStr">
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="20" t="inlineStr">
         <is>
           <t>• Workload Efficiency Score:</t>
         </is>
       </c>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="21" t="inlineStr">
-        <is>
-          <t>97.3% (High Contact Demand)</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
-      <c r="H26" s="4" t="n"/>
-      <c r="I26" s="4" t="n"/>
-      <c r="J26" s="4" t="n"/>
-      <c r="K26" s="4" t="n"/>
-      <c r="L26" s="4" t="n"/>
-      <c r="M26" s="4" t="n"/>
-      <c r="N26" s="4" t="n"/>
-      <c r="O26" s="4" t="n"/>
-      <c r="P26" s="4" t="n"/>
-      <c r="Q26" s="4" t="n"/>
-      <c r="R26" s="4" t="n"/>
-      <c r="S26" s="4" t="n"/>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="20" t="inlineStr">
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="n"/>
+      <c r="D36" s="4" t="n"/>
+      <c r="E36" s="21" t="inlineStr">
+        <is>
+          <t>25.0% (Critical Overload (Faculty Deficit))</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="n"/>
+      <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
+      <c r="I36" s="4" t="n"/>
+      <c r="J36" s="4" t="n"/>
+      <c r="K36" s="4" t="n"/>
+      <c r="L36" s="4" t="n"/>
+      <c r="M36" s="4" t="n"/>
+      <c r="N36" s="4" t="n"/>
+      <c r="O36" s="4" t="n"/>
+      <c r="P36" s="4" t="n"/>
+      <c r="Q36" s="4" t="n"/>
+      <c r="R36" s="4" t="n"/>
+      <c r="S36" s="4" t="n"/>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="20" t="inlineStr">
         <is>
           <t>• Available Faculty Capacity:</t>
         </is>
       </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="21" t="inlineStr">
-        <is>
-          <t>54 faculty × 15.0h = 810.0 faculty-hours available</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
-      <c r="I27" s="4" t="n"/>
-      <c r="J27" s="4" t="n"/>
-      <c r="K27" s="4" t="n"/>
-      <c r="L27" s="4" t="n"/>
-      <c r="M27" s="4" t="n"/>
-      <c r="N27" s="4" t="n"/>
-      <c r="O27" s="4" t="n"/>
-      <c r="P27" s="4" t="n"/>
-      <c r="Q27" s="4" t="n"/>
-      <c r="R27" s="4" t="n"/>
-      <c r="S27" s="4" t="n"/>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="20" t="inlineStr">
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="n"/>
+      <c r="D37" s="4" t="n"/>
+      <c r="E37" s="21" t="inlineStr">
+        <is>
+          <t>34 faculty × 15.0h = 510.0 faculty-hours available</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="4" t="n"/>
+      <c r="K37" s="4" t="n"/>
+      <c r="L37" s="4" t="n"/>
+      <c r="M37" s="4" t="n"/>
+      <c r="N37" s="4" t="n"/>
+      <c r="O37" s="4" t="n"/>
+      <c r="P37" s="4" t="n"/>
+      <c r="Q37" s="4" t="n"/>
+      <c r="R37" s="4" t="n"/>
+      <c r="S37" s="4" t="n"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="20" t="inlineStr">
         <is>
           <t>• Capacity Utilization Rate:</t>
         </is>
       </c>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="21" t="inlineStr">
-        <is>
-          <t>106.7% of total department capacity demand</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
-      <c r="H28" s="4" t="n"/>
-      <c r="I28" s="4" t="n"/>
-      <c r="J28" s="4" t="n"/>
-      <c r="K28" s="4" t="n"/>
-      <c r="L28" s="4" t="n"/>
-      <c r="M28" s="4" t="n"/>
-      <c r="N28" s="4" t="n"/>
-      <c r="O28" s="4" t="n"/>
-      <c r="P28" s="4" t="n"/>
-      <c r="Q28" s="4" t="n"/>
-      <c r="R28" s="4" t="n"/>
-      <c r="S28" s="4" t="n"/>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="20" t="inlineStr">
+      <c r="B38" s="4" t="n"/>
+      <c r="C38" s="4" t="n"/>
+      <c r="D38" s="4" t="n"/>
+      <c r="E38" s="21" t="inlineStr">
+        <is>
+          <t>392.9% of total department capacity demand</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="n"/>
+      <c r="G38" s="4" t="n"/>
+      <c r="H38" s="4" t="n"/>
+      <c r="I38" s="4" t="n"/>
+      <c r="J38" s="4" t="n"/>
+      <c r="K38" s="4" t="n"/>
+      <c r="L38" s="4" t="n"/>
+      <c r="M38" s="4" t="n"/>
+      <c r="N38" s="4" t="n"/>
+      <c r="O38" s="4" t="n"/>
+      <c r="P38" s="4" t="n"/>
+      <c r="Q38" s="4" t="n"/>
+      <c r="R38" s="4" t="n"/>
+      <c r="S38" s="4" t="n"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="20" t="inlineStr">
         <is>
           <t>• Faculty Headcount Balance:</t>
         </is>
       </c>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="21" t="inlineStr">
-        <is>
-          <t>Needed: 57.6 | Available: 54 | Deficit: -3.6 faculty</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
-      <c r="H29" s="4" t="n"/>
-      <c r="I29" s="4" t="n"/>
-      <c r="J29" s="4" t="n"/>
-      <c r="K29" s="4" t="n"/>
-      <c r="L29" s="4" t="n"/>
-      <c r="M29" s="4" t="n"/>
-      <c r="N29" s="4" t="n"/>
-      <c r="O29" s="4" t="n"/>
-      <c r="P29" s="4" t="n"/>
-      <c r="Q29" s="4" t="n"/>
-      <c r="R29" s="4" t="n"/>
-      <c r="S29" s="4" t="n"/>
+      <c r="B39" s="4" t="n"/>
+      <c r="C39" s="4" t="n"/>
+      <c r="D39" s="4" t="n"/>
+      <c r="E39" s="21" t="inlineStr">
+        <is>
+          <t>Needed: 133.6 | Available: 34 | Deficit: -99.6 faculty</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="n"/>
+      <c r="G39" s="4" t="n"/>
+      <c r="H39" s="4" t="n"/>
+      <c r="I39" s="4" t="n"/>
+      <c r="J39" s="4" t="n"/>
+      <c r="K39" s="4" t="n"/>
+      <c r="L39" s="4" t="n"/>
+      <c r="M39" s="4" t="n"/>
+      <c r="N39" s="4" t="n"/>
+      <c r="O39" s="4" t="n"/>
+      <c r="P39" s="4" t="n"/>
+      <c r="Q39" s="4" t="n"/>
+      <c r="R39" s="4" t="n"/>
+      <c r="S39" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="E29:S29"/>
     <mergeCell ref="Q5:S5"/>
-    <mergeCell ref="E20:S20"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="E28:S28"/>
-    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="E38:S38"/>
+    <mergeCell ref="A38:D38"/>
     <mergeCell ref="Q4:S4"/>
-    <mergeCell ref="A29:D29"/>
     <mergeCell ref="J4:L4"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A19:S19"/>
+    <mergeCell ref="E31:S31"/>
+    <mergeCell ref="A35:S35"/>
+    <mergeCell ref="A29:S29"/>
+    <mergeCell ref="E30:S30"/>
+    <mergeCell ref="A31:D31"/>
     <mergeCell ref="M4:P4"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="G5:I5"/>
+    <mergeCell ref="A32:D32"/>
     <mergeCell ref="D4:F4"/>
-    <mergeCell ref="E27:S27"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="E36:S36"/>
+    <mergeCell ref="A39:D39"/>
     <mergeCell ref="G4:I4"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="E26:S26"/>
+    <mergeCell ref="A36:D36"/>
     <mergeCell ref="M5:P5"/>
     <mergeCell ref="D5:F5"/>
+    <mergeCell ref="E32:S32"/>
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="E22:S22"/>
-    <mergeCell ref="E21:S21"/>
+    <mergeCell ref="E37:S37"/>
     <mergeCell ref="J5:L5"/>
-    <mergeCell ref="A25:S25"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="E23:S23"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="E33:S33"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="E39:S39"/>
     <mergeCell ref="A2:S2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1731,22 +2361,22 @@
         </is>
       </c>
       <c r="C4" s="10" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D4" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="E4" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="E4" s="10" t="n">
-        <v>0</v>
-      </c>
       <c r="F4" s="10" t="n">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="G4" s="12" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="H4" s="12" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -1759,22 +2389,22 @@
         </is>
       </c>
       <c r="C5" s="13" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D5" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="E5" s="13" t="n">
         <v>24</v>
       </c>
-      <c r="E5" s="13" t="n">
-        <v>0</v>
-      </c>
       <c r="F5" s="13" t="n">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="G5" s="15" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>144</v>
+        <v>334</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -1787,22 +2417,22 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D6" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="E6" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="E6" s="10" t="n">
-        <v>0</v>
-      </c>
       <c r="F6" s="10" t="n">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="G6" s="12" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="H6" s="12" t="n">
-        <v>216</v>
+        <v>501</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -1815,22 +2445,22 @@
         </is>
       </c>
       <c r="C7" s="13" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D7" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="E7" s="13" t="n">
         <v>24</v>
       </c>
-      <c r="E7" s="13" t="n">
-        <v>0</v>
-      </c>
       <c r="F7" s="13" t="n">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="G7" s="15" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>288</v>
+        <v>668</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -1843,22 +2473,22 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D8" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="E8" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="E8" s="10" t="n">
-        <v>0</v>
-      </c>
       <c r="F8" s="10" t="n">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="H8" s="12" t="n">
-        <v>360</v>
+        <v>835</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -1871,22 +2501,22 @@
         </is>
       </c>
       <c r="C9" s="13" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D9" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="E9" s="13" t="n">
         <v>24</v>
       </c>
-      <c r="E9" s="13" t="n">
-        <v>0</v>
-      </c>
       <c r="F9" s="13" t="n">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="G9" s="15" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>432</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -1899,22 +2529,22 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D10" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="E10" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="E10" s="10" t="n">
-        <v>0</v>
-      </c>
       <c r="F10" s="10" t="n">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="H10" s="12" t="n">
-        <v>504</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -1927,22 +2557,22 @@
         </is>
       </c>
       <c r="C11" s="13" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D11" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="E11" s="13" t="n">
         <v>24</v>
       </c>
-      <c r="E11" s="13" t="n">
-        <v>0</v>
-      </c>
       <c r="F11" s="13" t="n">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="G11" s="15" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>576</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -1955,22 +2585,22 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D12" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="E12" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="E12" s="10" t="n">
-        <v>0</v>
-      </c>
       <c r="F12" s="10" t="n">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="H12" s="12" t="n">
-        <v>648</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -1983,22 +2613,22 @@
         </is>
       </c>
       <c r="C13" s="13" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D13" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="E13" s="13" t="n">
         <v>24</v>
       </c>
-      <c r="E13" s="13" t="n">
-        <v>0</v>
-      </c>
       <c r="F13" s="13" t="n">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="G13" s="15" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>720</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
@@ -2011,22 +2641,22 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D14" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="E14" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="E14" s="10" t="n">
-        <v>0</v>
-      </c>
       <c r="F14" s="10" t="n">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="G14" s="12" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>792</v>
+        <v>1837</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -2039,22 +2669,22 @@
         </is>
       </c>
       <c r="C15" s="13" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D15" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="E15" s="13" t="n">
         <v>24</v>
       </c>
-      <c r="E15" s="13" t="n">
-        <v>0</v>
-      </c>
       <c r="F15" s="13" t="n">
-        <v>48</v>
+        <v>108</v>
       </c>
       <c r="G15" s="15" t="n">
-        <v>72</v>
+        <v>167</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>864</v>
+        <v>2004</v>
       </c>
     </row>
   </sheetData>
@@ -2168,23 +2798,23 @@
       </c>
       <c r="E4" s="25" t="inlineStr">
         <is>
-          <t>72h</t>
+          <t>167h</t>
         </is>
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>864h</t>
+          <t>2004h</t>
         </is>
       </c>
       <c r="G4" s="25" t="n">
-        <v>57.6</v>
+        <v>133.6</v>
       </c>
       <c r="H4" s="25" t="n">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="I4" s="26" t="inlineStr">
         <is>
-          <t>-3.6 deficit</t>
+          <t>-99.6 deficit</t>
         </is>
       </c>
       <c r="J4" s="25" t="inlineStr">
@@ -2215,33 +2845,33 @@
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>56h</t>
+          <t>123h</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>672h</t>
+          <t>1476h</t>
         </is>
       </c>
       <c r="G5" s="13" t="n">
-        <v>44.8</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="H5" s="13" t="n">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
-          <t>+9.2 surplus</t>
+          <t>-64.4 deficit</t>
         </is>
       </c>
       <c r="J5" s="27" t="inlineStr">
         <is>
-          <t>192h</t>
+          <t>528h</t>
         </is>
       </c>
       <c r="K5" s="13" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>26.3%</t>
         </is>
       </c>
     </row>
@@ -2262,33 +2892,33 @@
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>56h</t>
+          <t>115h</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>672h</t>
+          <t>1380h</t>
         </is>
       </c>
       <c r="G6" s="10" t="n">
-        <v>44.8</v>
+        <v>92</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="I6" s="12" t="inlineStr">
         <is>
-          <t>+9.2 surplus</t>
+          <t>-58.0 deficit</t>
         </is>
       </c>
       <c r="J6" s="27" t="inlineStr">
         <is>
-          <t>192h</t>
+          <t>624h</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>22.2%</t>
+          <t>31.1%</t>
         </is>
       </c>
     </row>
@@ -2309,33 +2939,33 @@
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>40h</t>
+          <t>79h</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>480h</t>
+          <t>948h</t>
         </is>
       </c>
       <c r="G7" s="13" t="n">
-        <v>32</v>
+        <v>63.2</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>+22.0 surplus</t>
+          <t>-29.2 deficit</t>
         </is>
       </c>
       <c r="J7" s="27" t="inlineStr">
         <is>
-          <t>384h</t>
+          <t>1056h</t>
         </is>
       </c>
       <c r="K7" s="13" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>52.7%</t>
         </is>
       </c>
     </row>
@@ -2381,12 +3011,12 @@
       </c>
       <c r="C12" s="29" t="inlineStr">
         <is>
-          <t>9 faculty</t>
+          <t>20 faculty</t>
         </is>
       </c>
       <c r="D12" s="29" t="inlineStr">
         <is>
-          <t>108 hrs</t>
+          <t>240 hrs</t>
         </is>
       </c>
     </row>
@@ -2403,12 +3033,12 @@
       </c>
       <c r="C13" s="30" t="inlineStr">
         <is>
-          <t>14 faculty</t>
+          <t>33 faculty</t>
         </is>
       </c>
       <c r="D13" s="30" t="inlineStr">
         <is>
-          <t>196 hrs</t>
+          <t>462 hrs</t>
         </is>
       </c>
     </row>
@@ -2425,12 +3055,12 @@
       </c>
       <c r="C14" s="29" t="inlineStr">
         <is>
-          <t>35 faculty</t>
+          <t>81 faculty</t>
         </is>
       </c>
       <c r="D14" s="29" t="inlineStr">
         <is>
-          <t>560 hrs</t>
+          <t>1296 hrs</t>
         </is>
       </c>
     </row>

</xml_diff>